<commit_message>
Close out GS1 registration: bundles live in Data Hub, dupes archived, conflicts resolved
- Bundles registered 2026-07-03 with exact expected GTINs (362/379/386);
  regenerate gs1-import-corrected.xlsx without bundle rows or archived dupes
  (BUNDLES_REGISTERED / SKIP_GTINS flags in build-gs1-import.py)
- Shade conflict review closed: GS1 wins all 74 rows, zero overrides
- Duplicate GTINs 850066107188/195 archived in Data Hub; docs updated
- AGENTS.md + skill reflect single remaining task: bulk name-correction import

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/DISURI Beauty/product-master/gs1-import-corrected.xlsx
+++ b/DISURI Beauty/product-master/gs1-import-corrected.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO240"/>
+  <dimension ref="A1:AO235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
   <cols>
     <col width="19" customWidth="1" style="1" min="1" max="1"/>
@@ -27742,13 +27742,13 @@
       </c>
       <c r="B220" s="1" t="inlineStr">
         <is>
-          <t>00850066107188</t>
+          <t>00850066107201</t>
         </is>
       </c>
       <c r="C220" s="1" t="inlineStr"/>
       <c r="D220" s="1" t="inlineStr">
         <is>
-          <t>850066107188</t>
+          <t>850066107201</t>
         </is>
       </c>
       <c r="E220" s="1" t="inlineStr"/>
@@ -27764,7 +27764,7 @@
       </c>
       <c r="H220" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Triple Collagen Firming Essence</t>
+          <t>DISURI Beauty Shimmer Blast Lip Gloss - Green Crush (S71)</t>
         </is>
       </c>
       <c r="I220" s="1" t="inlineStr">
@@ -27802,7 +27802,11 @@
       <c r="Q220" s="1" t="inlineStr"/>
       <c r="S220" s="1" t="inlineStr"/>
       <c r="T220" s="1" t="inlineStr"/>
-      <c r="V220" s="1" t="inlineStr"/>
+      <c r="V220" s="1" t="inlineStr">
+        <is>
+          <t>S71</t>
+        </is>
+      </c>
       <c r="W220" s="1" t="inlineStr"/>
       <c r="X220" s="1" t="inlineStr"/>
       <c r="Y220" s="1" t="inlineStr"/>
@@ -27820,10 +27824,14 @@
       <c r="AK220" s="2" t="inlineStr"/>
       <c r="AL220" s="1" t="inlineStr"/>
       <c r="AM220" s="1" t="inlineStr"/>
-      <c r="AN220" s="1" t="inlineStr"/>
+      <c r="AN220" s="1" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
       <c r="AO220" s="1" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>2025-01-15</t>
         </is>
       </c>
     </row>
@@ -27835,13 +27843,13 @@
       </c>
       <c r="B221" s="1" t="inlineStr">
         <is>
-          <t>00850066107195</t>
+          <t>00850066107218</t>
         </is>
       </c>
       <c r="C221" s="1" t="inlineStr"/>
       <c r="D221" s="1" t="inlineStr">
         <is>
-          <t>850066107195</t>
+          <t>850066107218</t>
         </is>
       </c>
       <c r="E221" s="1" t="inlineStr"/>
@@ -27857,7 +27865,7 @@
       </c>
       <c r="H221" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Ultra Plumping Blast Lip Gloss - Mango (8)</t>
+          <t>DISURI Beauty Color Pop Lip Liner - Berry Temptation (LLBT10)</t>
         </is>
       </c>
       <c r="I221" s="1" t="inlineStr">
@@ -27897,7 +27905,7 @@
       <c r="T221" s="1" t="inlineStr"/>
       <c r="V221" s="1" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>LLBT10</t>
         </is>
       </c>
       <c r="W221" s="1" t="inlineStr"/>
@@ -27917,10 +27925,14 @@
       <c r="AK221" s="2" t="inlineStr"/>
       <c r="AL221" s="1" t="inlineStr"/>
       <c r="AM221" s="1" t="inlineStr"/>
-      <c r="AN221" s="1" t="inlineStr"/>
+      <c r="AN221" s="1" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
       <c r="AO221" s="1" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>2025-01-16</t>
         </is>
       </c>
     </row>
@@ -27932,13 +27944,13 @@
       </c>
       <c r="B222" s="1" t="inlineStr">
         <is>
-          <t>00850066107201</t>
+          <t>00850066107225</t>
         </is>
       </c>
       <c r="C222" s="1" t="inlineStr"/>
       <c r="D222" s="1" t="inlineStr">
         <is>
-          <t>850066107201</t>
+          <t>850066107225</t>
         </is>
       </c>
       <c r="E222" s="1" t="inlineStr"/>
@@ -27954,7 +27966,7 @@
       </c>
       <c r="H222" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Shimmer Blast Lip Gloss - Green Crush (S71)</t>
+          <t>DISURI Beauty Matte &amp; Glam Collection</t>
         </is>
       </c>
       <c r="I222" s="1" t="inlineStr">
@@ -27992,11 +28004,7 @@
       <c r="Q222" s="1" t="inlineStr"/>
       <c r="S222" s="1" t="inlineStr"/>
       <c r="T222" s="1" t="inlineStr"/>
-      <c r="V222" s="1" t="inlineStr">
-        <is>
-          <t>S71</t>
-        </is>
-      </c>
+      <c r="V222" s="1" t="inlineStr"/>
       <c r="W222" s="1" t="inlineStr"/>
       <c r="X222" s="1" t="inlineStr"/>
       <c r="Y222" s="1" t="inlineStr"/>
@@ -28021,7 +28029,7 @@
       </c>
       <c r="AO222" s="1" t="inlineStr">
         <is>
-          <t>2025-01-15</t>
+          <t>2024-10-01</t>
         </is>
       </c>
     </row>
@@ -28033,13 +28041,13 @@
       </c>
       <c r="B223" s="1" t="inlineStr">
         <is>
-          <t>00850066107218</t>
+          <t>00850066107232</t>
         </is>
       </c>
       <c r="C223" s="1" t="inlineStr"/>
       <c r="D223" s="1" t="inlineStr">
         <is>
-          <t>850066107218</t>
+          <t>850066107232</t>
         </is>
       </c>
       <c r="E223" s="1" t="inlineStr"/>
@@ -28055,7 +28063,7 @@
       </c>
       <c r="H223" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Color Pop Lip Liner - Berry Temptation (LLBT10)</t>
+          <t>DISURI Beauty Matte &amp; Glow Collection</t>
         </is>
       </c>
       <c r="I223" s="1" t="inlineStr">
@@ -28093,11 +28101,7 @@
       <c r="Q223" s="1" t="inlineStr"/>
       <c r="S223" s="1" t="inlineStr"/>
       <c r="T223" s="1" t="inlineStr"/>
-      <c r="V223" s="1" t="inlineStr">
-        <is>
-          <t>LLBT10</t>
-        </is>
-      </c>
+      <c r="V223" s="1" t="inlineStr"/>
       <c r="W223" s="1" t="inlineStr"/>
       <c r="X223" s="1" t="inlineStr"/>
       <c r="Y223" s="1" t="inlineStr"/>
@@ -28122,7 +28126,7 @@
       </c>
       <c r="AO223" s="1" t="inlineStr">
         <is>
-          <t>2025-01-16</t>
+          <t>2024-10-01</t>
         </is>
       </c>
     </row>
@@ -28134,13 +28138,13 @@
       </c>
       <c r="B224" s="1" t="inlineStr">
         <is>
-          <t>00850066107225</t>
+          <t>00850066107249</t>
         </is>
       </c>
       <c r="C224" s="1" t="inlineStr"/>
       <c r="D224" s="1" t="inlineStr">
         <is>
-          <t>850066107225</t>
+          <t>850066107249</t>
         </is>
       </c>
       <c r="E224" s="1" t="inlineStr"/>
@@ -28156,7 +28160,7 @@
       </c>
       <c r="H224" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Matte &amp; Glam Collection</t>
+          <t>DISURI Beauty Matte Addict Collection</t>
         </is>
       </c>
       <c r="I224" s="1" t="inlineStr">
@@ -28219,7 +28223,7 @@
       </c>
       <c r="AO224" s="1" t="inlineStr">
         <is>
-          <t>2024-10-01</t>
+          <t>2024-10-02</t>
         </is>
       </c>
     </row>
@@ -28231,19 +28235,19 @@
       </c>
       <c r="B225" s="1" t="inlineStr">
         <is>
-          <t>00850066107232</t>
+          <t>00850066107256</t>
         </is>
       </c>
       <c r="C225" s="1" t="inlineStr"/>
       <c r="D225" s="1" t="inlineStr">
         <is>
-          <t>850066107232</t>
+          <t>850066107256</t>
         </is>
       </c>
       <c r="E225" s="1" t="inlineStr"/>
       <c r="F225" s="1" t="inlineStr">
         <is>
-          <t>DISURI BEAUTY</t>
+          <t>DISURI Beauty</t>
         </is>
       </c>
       <c r="G225" s="1" t="inlineStr">
@@ -28253,7 +28257,7 @@
       </c>
       <c r="H225" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Matte &amp; Glow Collection</t>
+          <t>DISURI Beauty Cold Crush Shimmer Blast - 5-Pack</t>
         </is>
       </c>
       <c r="I225" s="1" t="inlineStr">
@@ -28316,7 +28320,7 @@
       </c>
       <c r="AO225" s="1" t="inlineStr">
         <is>
-          <t>2024-10-01</t>
+          <t>2024-10-07</t>
         </is>
       </c>
     </row>
@@ -28328,13 +28332,13 @@
       </c>
       <c r="B226" s="1" t="inlineStr">
         <is>
-          <t>00850066107249</t>
+          <t>00850066107263</t>
         </is>
       </c>
       <c r="C226" s="1" t="inlineStr"/>
       <c r="D226" s="1" t="inlineStr">
         <is>
-          <t>850066107249</t>
+          <t>850066107263</t>
         </is>
       </c>
       <c r="E226" s="1" t="inlineStr"/>
@@ -28350,7 +28354,7 @@
       </c>
       <c r="H226" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Matte Addict Collection</t>
+          <t>DISURI Beauty Candy Crush Collection</t>
         </is>
       </c>
       <c r="I226" s="1" t="inlineStr">
@@ -28413,7 +28417,7 @@
       </c>
       <c r="AO226" s="1" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>2024-10-07</t>
         </is>
       </c>
     </row>
@@ -28425,13 +28429,13 @@
       </c>
       <c r="B227" s="1" t="inlineStr">
         <is>
-          <t>00850066107256</t>
+          <t>00850066107270</t>
         </is>
       </c>
       <c r="C227" s="1" t="inlineStr"/>
       <c r="D227" s="1" t="inlineStr">
         <is>
-          <t>850066107256</t>
+          <t>850066107270</t>
         </is>
       </c>
       <c r="E227" s="1" t="inlineStr"/>
@@ -28447,7 +28451,7 @@
       </c>
       <c r="H227" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Cold Crush Shimmer Blast - 5-Pack</t>
+          <t>DISURI Beauty Shimmer &amp; Glam Collection</t>
         </is>
       </c>
       <c r="I227" s="1" t="inlineStr">
@@ -28522,19 +28526,19 @@
       </c>
       <c r="B228" s="1" t="inlineStr">
         <is>
-          <t>00850066107263</t>
+          <t>00850066107287</t>
         </is>
       </c>
       <c r="C228" s="1" t="inlineStr"/>
       <c r="D228" s="1" t="inlineStr">
         <is>
-          <t>850066107263</t>
+          <t>850066107287</t>
         </is>
       </c>
       <c r="E228" s="1" t="inlineStr"/>
       <c r="F228" s="1" t="inlineStr">
         <is>
-          <t>DISURI BEAUTY</t>
+          <t>DISURI Beauty</t>
         </is>
       </c>
       <c r="G228" s="1" t="inlineStr">
@@ -28544,7 +28548,7 @@
       </c>
       <c r="H228" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Candy Crush Collection</t>
+          <t>DISURI Beauty Pink Berry Diamonds Collection</t>
         </is>
       </c>
       <c r="I228" s="1" t="inlineStr">
@@ -28619,13 +28623,13 @@
       </c>
       <c r="B229" s="1" t="inlineStr">
         <is>
-          <t>00850066107270</t>
+          <t>00850066107294</t>
         </is>
       </c>
       <c r="C229" s="1" t="inlineStr"/>
       <c r="D229" s="1" t="inlineStr">
         <is>
-          <t>850066107270</t>
+          <t>850066107294</t>
         </is>
       </c>
       <c r="E229" s="1" t="inlineStr"/>
@@ -28641,7 +28645,7 @@
       </c>
       <c r="H229" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Shimmer &amp; Glam Collection</t>
+          <t>DISURI Beauty Cold Crush Shimmer Blast - 10-Pack</t>
         </is>
       </c>
       <c r="I229" s="1" t="inlineStr">
@@ -28716,13 +28720,13 @@
       </c>
       <c r="B230" s="1" t="inlineStr">
         <is>
-          <t>00850066107287</t>
+          <t>00850066107300</t>
         </is>
       </c>
       <c r="C230" s="1" t="inlineStr"/>
       <c r="D230" s="1" t="inlineStr">
         <is>
-          <t>850066107287</t>
+          <t>850066107300</t>
         </is>
       </c>
       <c r="E230" s="1" t="inlineStr"/>
@@ -28738,7 +28742,7 @@
       </c>
       <c r="H230" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Pink Berry Diamonds Collection</t>
+          <t>DISURI Beauty Cold Crush Shimmer Blast - 3-Pack</t>
         </is>
       </c>
       <c r="I230" s="1" t="inlineStr">
@@ -28801,7 +28805,7 @@
       </c>
       <c r="AO230" s="1" t="inlineStr">
         <is>
-          <t>2024-10-07</t>
+          <t>2024-10-10</t>
         </is>
       </c>
     </row>
@@ -28813,13 +28817,13 @@
       </c>
       <c r="B231" s="1" t="inlineStr">
         <is>
-          <t>00850066107294</t>
+          <t>00850066107317</t>
         </is>
       </c>
       <c r="C231" s="1" t="inlineStr"/>
       <c r="D231" s="1" t="inlineStr">
         <is>
-          <t>850066107294</t>
+          <t>850066107317</t>
         </is>
       </c>
       <c r="E231" s="1" t="inlineStr"/>
@@ -28835,7 +28839,7 @@
       </c>
       <c r="H231" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Cold Crush Shimmer Blast - 10-Pack</t>
+          <t>DISURI Beauty Shimmer Blast Lip Gloss - Sunset Glow</t>
         </is>
       </c>
       <c r="I231" s="1" t="inlineStr">
@@ -28898,7 +28902,7 @@
       </c>
       <c r="AO231" s="1" t="inlineStr">
         <is>
-          <t>2024-10-07</t>
+          <t>2024-11-06</t>
         </is>
       </c>
     </row>
@@ -28910,13 +28914,13 @@
       </c>
       <c r="B232" s="1" t="inlineStr">
         <is>
-          <t>00850066107300</t>
+          <t>00850066107324</t>
         </is>
       </c>
       <c r="C232" s="1" t="inlineStr"/>
       <c r="D232" s="1" t="inlineStr">
         <is>
-          <t>850066107300</t>
+          <t>850066107324</t>
         </is>
       </c>
       <c r="E232" s="1" t="inlineStr"/>
@@ -28932,7 +28936,7 @@
       </c>
       <c r="H232" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Cold Crush Shimmer Blast - 3-Pack</t>
+          <t>DISURI Beauty Color Pop Lip Liner - Rouge Rush Berry (LLRR12)</t>
         </is>
       </c>
       <c r="I232" s="1" t="inlineStr">
@@ -28970,7 +28974,11 @@
       <c r="Q232" s="1" t="inlineStr"/>
       <c r="S232" s="1" t="inlineStr"/>
       <c r="T232" s="1" t="inlineStr"/>
-      <c r="V232" s="1" t="inlineStr"/>
+      <c r="V232" s="1" t="inlineStr">
+        <is>
+          <t>LLRR12</t>
+        </is>
+      </c>
       <c r="W232" s="1" t="inlineStr"/>
       <c r="X232" s="1" t="inlineStr"/>
       <c r="Y232" s="1" t="inlineStr"/>
@@ -28995,7 +29003,7 @@
       </c>
       <c r="AO232" s="1" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>2025-01-16</t>
         </is>
       </c>
     </row>
@@ -29007,13 +29015,13 @@
       </c>
       <c r="B233" s="1" t="inlineStr">
         <is>
-          <t>00850066107317</t>
+          <t>00850066107331</t>
         </is>
       </c>
       <c r="C233" s="1" t="inlineStr"/>
       <c r="D233" s="1" t="inlineStr">
         <is>
-          <t>850066107317</t>
+          <t>850066107331</t>
         </is>
       </c>
       <c r="E233" s="1" t="inlineStr"/>
@@ -29029,7 +29037,7 @@
       </c>
       <c r="H233" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Shimmer Blast Lip Gloss - Sunset Glow</t>
+          <t>DISURI Beauty Color Pop Lip Liner - Sunset Passion (LLSP8)</t>
         </is>
       </c>
       <c r="I233" s="1" t="inlineStr">
@@ -29067,7 +29075,11 @@
       <c r="Q233" s="1" t="inlineStr"/>
       <c r="S233" s="1" t="inlineStr"/>
       <c r="T233" s="1" t="inlineStr"/>
-      <c r="V233" s="1" t="inlineStr"/>
+      <c r="V233" s="1" t="inlineStr">
+        <is>
+          <t>LLSP8</t>
+        </is>
+      </c>
       <c r="W233" s="1" t="inlineStr"/>
       <c r="X233" s="1" t="inlineStr"/>
       <c r="Y233" s="1" t="inlineStr"/>
@@ -29092,7 +29104,7 @@
       </c>
       <c r="AO233" s="1" t="inlineStr">
         <is>
-          <t>2024-11-06</t>
+          <t>2025-01-16</t>
         </is>
       </c>
     </row>
@@ -29104,13 +29116,13 @@
       </c>
       <c r="B234" s="1" t="inlineStr">
         <is>
-          <t>00850066107324</t>
+          <t>00850066107348</t>
         </is>
       </c>
       <c r="C234" s="1" t="inlineStr"/>
       <c r="D234" s="1" t="inlineStr">
         <is>
-          <t>850066107324</t>
+          <t>850066107348</t>
         </is>
       </c>
       <c r="E234" s="1" t="inlineStr"/>
@@ -29126,7 +29138,7 @@
       </c>
       <c r="H234" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Color Pop Lip Liner - Rouge Rush Berry (LLRR12)</t>
+          <t>DISURI Beauty Color Pop Lip Liner - Blush Blossom (LLBB6)</t>
         </is>
       </c>
       <c r="I234" s="1" t="inlineStr">
@@ -29166,7 +29178,7 @@
       <c r="T234" s="1" t="inlineStr"/>
       <c r="V234" s="1" t="inlineStr">
         <is>
-          <t>LLRR12</t>
+          <t>LLBB6</t>
         </is>
       </c>
       <c r="W234" s="1" t="inlineStr"/>
@@ -29205,13 +29217,13 @@
       </c>
       <c r="B235" s="1" t="inlineStr">
         <is>
-          <t>00850066107331</t>
+          <t>00850066107355</t>
         </is>
       </c>
       <c r="C235" s="1" t="inlineStr"/>
       <c r="D235" s="1" t="inlineStr">
         <is>
-          <t>850066107331</t>
+          <t>850066107355</t>
         </is>
       </c>
       <c r="E235" s="1" t="inlineStr"/>
@@ -29227,7 +29239,7 @@
       </c>
       <c r="H235" s="1" t="inlineStr">
         <is>
-          <t>DISURI Beauty Color Pop Lip Liner - Sunset Passion (LLSP8)</t>
+          <t>DISURI Beauty Color Pop Lip Liner - Nude Mood (LLNM)</t>
         </is>
       </c>
       <c r="I235" s="1" t="inlineStr">
@@ -29267,7 +29279,7 @@
       <c r="T235" s="1" t="inlineStr"/>
       <c r="V235" s="1" t="inlineStr">
         <is>
-          <t>LLSP8</t>
+          <t>LLNM</t>
         </is>
       </c>
       <c r="W235" s="1" t="inlineStr"/>
@@ -29298,517 +29310,8 @@
         </is>
       </c>
     </row>
-    <row r="236" ht="12.75" customHeight="1">
-      <c r="A236" s="1" t="inlineStr">
-        <is>
-          <t>0850066107</t>
-        </is>
-      </c>
-      <c r="B236" s="1" t="inlineStr">
-        <is>
-          <t>00850066107348</t>
-        </is>
-      </c>
-      <c r="C236" s="1" t="inlineStr"/>
-      <c r="D236" s="1" t="inlineStr">
-        <is>
-          <t>850066107348</t>
-        </is>
-      </c>
-      <c r="E236" s="1" t="inlineStr"/>
-      <c r="F236" s="1" t="inlineStr">
-        <is>
-          <t>DISURI Beauty</t>
-        </is>
-      </c>
-      <c r="G236" s="1" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="H236" s="1" t="inlineStr">
-        <is>
-          <t>DISURI Beauty Color Pop Lip Liner - Blush Blossom (LLBB6)</t>
-        </is>
-      </c>
-      <c r="I236" s="1" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="J236" s="1" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="K236" s="1" t="inlineStr">
-        <is>
-          <t>Each</t>
-        </is>
-      </c>
-      <c r="L236" s="1" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M236" s="1" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N236" s="1" t="inlineStr">
-        <is>
-          <t>In Use</t>
-        </is>
-      </c>
-      <c r="O236" s="1" t="inlineStr"/>
-      <c r="P236" s="1" t="inlineStr"/>
-      <c r="Q236" s="1" t="inlineStr"/>
-      <c r="S236" s="1" t="inlineStr"/>
-      <c r="T236" s="1" t="inlineStr"/>
-      <c r="V236" s="1" t="inlineStr">
-        <is>
-          <t>LLBB6</t>
-        </is>
-      </c>
-      <c r="W236" s="1" t="inlineStr"/>
-      <c r="X236" s="1" t="inlineStr"/>
-      <c r="Y236" s="1" t="inlineStr"/>
-      <c r="Z236" s="1" t="inlineStr"/>
-      <c r="AA236" s="1" t="inlineStr"/>
-      <c r="AB236" s="1" t="inlineStr"/>
-      <c r="AC236" s="1" t="inlineStr"/>
-      <c r="AD236" s="1" t="inlineStr"/>
-      <c r="AE236" s="1" t="inlineStr"/>
-      <c r="AF236" s="1" t="inlineStr"/>
-      <c r="AG236" s="1" t="inlineStr"/>
-      <c r="AH236" s="1" t="inlineStr"/>
-      <c r="AI236" s="1" t="inlineStr"/>
-      <c r="AJ236" s="1" t="inlineStr"/>
-      <c r="AK236" s="2" t="inlineStr"/>
-      <c r="AL236" s="1" t="inlineStr"/>
-      <c r="AM236" s="1" t="inlineStr"/>
-      <c r="AN236" s="1" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="AO236" s="1" t="inlineStr">
-        <is>
-          <t>2025-01-16</t>
-        </is>
-      </c>
-    </row>
-    <row r="237" ht="12.75" customHeight="1">
-      <c r="A237" s="1" t="inlineStr">
-        <is>
-          <t>0850066107</t>
-        </is>
-      </c>
-      <c r="B237" s="1" t="inlineStr">
-        <is>
-          <t>00850066107355</t>
-        </is>
-      </c>
-      <c r="C237" s="1" t="inlineStr"/>
-      <c r="D237" s="1" t="inlineStr">
-        <is>
-          <t>850066107355</t>
-        </is>
-      </c>
-      <c r="E237" s="1" t="inlineStr"/>
-      <c r="F237" s="1" t="inlineStr">
-        <is>
-          <t>DISURI Beauty</t>
-        </is>
-      </c>
-      <c r="G237" s="1" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="H237" s="1" t="inlineStr">
-        <is>
-          <t>DISURI Beauty Color Pop Lip Liner - Nude Mood (LLNM)</t>
-        </is>
-      </c>
-      <c r="I237" s="1" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="J237" s="1" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="K237" s="1" t="inlineStr">
-        <is>
-          <t>Each</t>
-        </is>
-      </c>
-      <c r="L237" s="1" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M237" s="1" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N237" s="1" t="inlineStr">
-        <is>
-          <t>In Use</t>
-        </is>
-      </c>
-      <c r="O237" s="1" t="inlineStr"/>
-      <c r="P237" s="1" t="inlineStr"/>
-      <c r="Q237" s="1" t="inlineStr"/>
-      <c r="S237" s="1" t="inlineStr"/>
-      <c r="T237" s="1" t="inlineStr"/>
-      <c r="V237" s="1" t="inlineStr">
-        <is>
-          <t>LLNM</t>
-        </is>
-      </c>
-      <c r="W237" s="1" t="inlineStr"/>
-      <c r="X237" s="1" t="inlineStr"/>
-      <c r="Y237" s="1" t="inlineStr"/>
-      <c r="Z237" s="1" t="inlineStr"/>
-      <c r="AA237" s="1" t="inlineStr"/>
-      <c r="AB237" s="1" t="inlineStr"/>
-      <c r="AC237" s="1" t="inlineStr"/>
-      <c r="AD237" s="1" t="inlineStr"/>
-      <c r="AE237" s="1" t="inlineStr"/>
-      <c r="AF237" s="1" t="inlineStr"/>
-      <c r="AG237" s="1" t="inlineStr"/>
-      <c r="AH237" s="1" t="inlineStr"/>
-      <c r="AI237" s="1" t="inlineStr"/>
-      <c r="AJ237" s="1" t="inlineStr"/>
-      <c r="AK237" s="2" t="inlineStr"/>
-      <c r="AL237" s="1" t="inlineStr"/>
-      <c r="AM237" s="1" t="inlineStr"/>
-      <c r="AN237" s="1" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="AO237" s="1" t="inlineStr">
-        <is>
-          <t>2025-01-16</t>
-        </is>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" t="inlineStr">
-        <is>
-          <t>0850066107</t>
-        </is>
-      </c>
-      <c r="B238" t="inlineStr">
-        <is>
-          <t>00850066107362</t>
-        </is>
-      </c>
-      <c r="C238" t="inlineStr"/>
-      <c r="D238" t="inlineStr">
-        <is>
-          <t>850066107362</t>
-        </is>
-      </c>
-      <c r="E238" t="inlineStr"/>
-      <c r="F238" t="inlineStr">
-        <is>
-          <t>DISURI BEAUTY</t>
-        </is>
-      </c>
-      <c r="G238" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="H238" t="inlineStr">
-        <is>
-          <t>DISURI Beauty The Complete DISURI System - 3-Step Korean Skincare Routine</t>
-        </is>
-      </c>
-      <c r="I238" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="J238" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="K238" t="inlineStr">
-        <is>
-          <t>Each</t>
-        </is>
-      </c>
-      <c r="L238" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M238" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N238" t="inlineStr">
-        <is>
-          <t>In Use</t>
-        </is>
-      </c>
-      <c r="O238" t="inlineStr"/>
-      <c r="P238" t="inlineStr"/>
-      <c r="Q238" t="inlineStr"/>
-      <c r="R238" t="inlineStr"/>
-      <c r="S238" t="inlineStr"/>
-      <c r="T238" t="inlineStr"/>
-      <c r="U238" t="inlineStr"/>
-      <c r="V238" t="inlineStr">
-        <is>
-          <t>DIS-SYS-COMPLETE</t>
-        </is>
-      </c>
-      <c r="W238" t="inlineStr"/>
-      <c r="X238" t="inlineStr"/>
-      <c r="Y238" t="inlineStr"/>
-      <c r="Z238" t="inlineStr"/>
-      <c r="AA238" t="inlineStr"/>
-      <c r="AB238" t="inlineStr"/>
-      <c r="AC238" t="inlineStr"/>
-      <c r="AD238" t="inlineStr"/>
-      <c r="AE238" t="inlineStr"/>
-      <c r="AF238" t="inlineStr"/>
-      <c r="AG238" t="inlineStr"/>
-      <c r="AH238" t="inlineStr"/>
-      <c r="AI238" t="inlineStr"/>
-      <c r="AJ238" t="inlineStr">
-        <is>
-          <t>99999999 - Temporary Classification</t>
-        </is>
-      </c>
-      <c r="AK238" t="inlineStr"/>
-      <c r="AL238" t="inlineStr"/>
-      <c r="AM238" t="inlineStr"/>
-      <c r="AN238" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="AO238" t="inlineStr"/>
-    </row>
-    <row r="239">
-      <c r="A239" t="inlineStr">
-        <is>
-          <t>0850066107</t>
-        </is>
-      </c>
-      <c r="B239" t="inlineStr">
-        <is>
-          <t>00850066107379</t>
-        </is>
-      </c>
-      <c r="C239" t="inlineStr"/>
-      <c r="D239" t="inlineStr">
-        <is>
-          <t>850066107379</t>
-        </is>
-      </c>
-      <c r="E239" t="inlineStr"/>
-      <c r="F239" t="inlineStr">
-        <is>
-          <t>DISURI BEAUTY</t>
-        </is>
-      </c>
-      <c r="G239" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="H239" t="inlineStr">
-        <is>
-          <t>DISURI Beauty The Anti-Aging Power Duo - Korean Skincare Set</t>
-        </is>
-      </c>
-      <c r="I239" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="J239" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="K239" t="inlineStr">
-        <is>
-          <t>Each</t>
-        </is>
-      </c>
-      <c r="L239" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M239" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N239" t="inlineStr">
-        <is>
-          <t>In Use</t>
-        </is>
-      </c>
-      <c r="O239" t="inlineStr"/>
-      <c r="P239" t="inlineStr"/>
-      <c r="Q239" t="inlineStr"/>
-      <c r="R239" t="inlineStr"/>
-      <c r="S239" t="inlineStr"/>
-      <c r="T239" t="inlineStr"/>
-      <c r="U239" t="inlineStr"/>
-      <c r="V239" t="inlineStr">
-        <is>
-          <t>DIS-SYS-AADUO</t>
-        </is>
-      </c>
-      <c r="W239" t="inlineStr"/>
-      <c r="X239" t="inlineStr"/>
-      <c r="Y239" t="inlineStr"/>
-      <c r="Z239" t="inlineStr"/>
-      <c r="AA239" t="inlineStr"/>
-      <c r="AB239" t="inlineStr"/>
-      <c r="AC239" t="inlineStr"/>
-      <c r="AD239" t="inlineStr"/>
-      <c r="AE239" t="inlineStr"/>
-      <c r="AF239" t="inlineStr"/>
-      <c r="AG239" t="inlineStr"/>
-      <c r="AH239" t="inlineStr"/>
-      <c r="AI239" t="inlineStr"/>
-      <c r="AJ239" t="inlineStr">
-        <is>
-          <t>99999999 - Temporary Classification</t>
-        </is>
-      </c>
-      <c r="AK239" t="inlineStr"/>
-      <c r="AL239" t="inlineStr"/>
-      <c r="AM239" t="inlineStr"/>
-      <c r="AN239" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="AO239" t="inlineStr"/>
-    </row>
-    <row r="240">
-      <c r="A240" t="inlineStr">
-        <is>
-          <t>0850066107</t>
-        </is>
-      </c>
-      <c r="B240" t="inlineStr">
-        <is>
-          <t>00850066107386</t>
-        </is>
-      </c>
-      <c r="C240" t="inlineStr"/>
-      <c r="D240" t="inlineStr">
-        <is>
-          <t>850066107386</t>
-        </is>
-      </c>
-      <c r="E240" t="inlineStr"/>
-      <c r="F240" t="inlineStr">
-        <is>
-          <t>DISURI BEAUTY</t>
-        </is>
-      </c>
-      <c r="G240" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="H240" t="inlineStr">
-        <is>
-          <t>DISURI Beauty The Barrier Rescue System - Korean Skincare Set</t>
-        </is>
-      </c>
-      <c r="I240" t="inlineStr">
-        <is>
-          <t>en</t>
-        </is>
-      </c>
-      <c r="J240" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="K240" t="inlineStr">
-        <is>
-          <t>Each</t>
-        </is>
-      </c>
-      <c r="L240" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M240" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N240" t="inlineStr">
-        <is>
-          <t>In Use</t>
-        </is>
-      </c>
-      <c r="O240" t="inlineStr"/>
-      <c r="P240" t="inlineStr"/>
-      <c r="Q240" t="inlineStr"/>
-      <c r="R240" t="inlineStr"/>
-      <c r="S240" t="inlineStr"/>
-      <c r="T240" t="inlineStr"/>
-      <c r="U240" t="inlineStr"/>
-      <c r="V240" t="inlineStr">
-        <is>
-          <t>DIS-SYS-BARRIER</t>
-        </is>
-      </c>
-      <c r="W240" t="inlineStr"/>
-      <c r="X240" t="inlineStr"/>
-      <c r="Y240" t="inlineStr"/>
-      <c r="Z240" t="inlineStr"/>
-      <c r="AA240" t="inlineStr"/>
-      <c r="AB240" t="inlineStr"/>
-      <c r="AC240" t="inlineStr"/>
-      <c r="AD240" t="inlineStr"/>
-      <c r="AE240" t="inlineStr"/>
-      <c r="AF240" t="inlineStr"/>
-      <c r="AG240" t="inlineStr"/>
-      <c r="AH240" t="inlineStr"/>
-      <c r="AI240" t="inlineStr"/>
-      <c r="AJ240" t="inlineStr">
-        <is>
-          <t>99999999 - Temporary Classification</t>
-        </is>
-      </c>
-      <c r="AK240" t="inlineStr"/>
-      <c r="AL240" t="inlineStr"/>
-      <c r="AM240" t="inlineStr"/>
-      <c r="AN240" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="AO240" t="inlineStr"/>
-    </row>
+    <row r="236" ht="12.75" customHeight="1"/>
+    <row r="237" ht="12.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>